<commit_message>
data sets -- main data extraction is sar_extraction but I think there's data missing. Caitlin to finish extraction
</commit_message>
<xml_diff>
--- a/data/data_extraction.xlsx
+++ b/data/data_extraction.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ginacuomo-dannenburg/Documents/code/bvd-contacts/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0DA2BF40-ABF4-B149-B2F7-244878D54DD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADE71FAE-DCB5-3B46-A22B-563BF0EC9C83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="160" yWindow="660" windowWidth="38080" windowHeight="22060" activeTab="1" xr2:uid="{A7CE7862-27C5-4847-9280-1126E71BA906}"/>
+    <workbookView xWindow="160" yWindow="660" windowWidth="38080" windowHeight="22060" xr2:uid="{A7CE7862-27C5-4847-9280-1126E71BA906}"/>
   </bookViews>
   <sheets>
     <sheet name="data_extraction" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="132">
   <si>
     <t>first_author</t>
   </si>
@@ -99,12 +99,6 @@
     <t>DOI</t>
   </si>
   <si>
-    <t>where was the study conducted? If it was in multiple locations, please separate with a ";"</t>
-  </si>
-  <si>
-    <t>where was the study conducted? If it was in multiple countries, please separate with a ";"</t>
-  </si>
-  <si>
     <t>study_design</t>
   </si>
   <si>
@@ -129,12 +123,6 @@
     <t xml:space="preserve">design of the study. Please do not extract the meta-analysis because we will bias the outputs </t>
   </si>
   <si>
-    <t xml:space="preserve">number of confirmed cases </t>
-  </si>
-  <si>
-    <t xml:space="preserve">number of contacts </t>
-  </si>
-  <si>
     <t>case_definition</t>
   </si>
   <si>
@@ -142,19 +130,337 @@
   </si>
   <si>
     <t>what is the outcome of the index case? E.g. are these only contacts from EVD patients who died, or if it has SAR split by outcome of the index please extract separately</t>
+  </si>
+  <si>
+    <t>total_contacts</t>
+  </si>
+  <si>
+    <t>number of confirmed cases satisfying the definition of a contact in this row</t>
+  </si>
+  <si>
+    <t>number of contacts satisfying the definition of a contact in this row</t>
+  </si>
+  <si>
+    <t>total number of contacts in the study across all definitions covered in this study</t>
+  </si>
+  <si>
+    <t>where was the study conducted? If it was in multiple locations, please separate with a ";". If data is disaggregated by location and/or country, please extract them separately</t>
+  </si>
+  <si>
+    <t>where was the study conducted? If it was in multiple countries, please separate with a ";". If data is disaggregated by location and/or country, please extract them separately</t>
+  </si>
+  <si>
+    <t>Baron</t>
+  </si>
+  <si>
+    <t>PMC2536233</t>
+  </si>
+  <si>
+    <t>Nzara; Yambio</t>
+  </si>
+  <si>
+    <t>Sudan (now South Sudan)</t>
+  </si>
+  <si>
+    <t>Concurrent and retrospective</t>
+  </si>
+  <si>
+    <t>direct contact</t>
+  </si>
+  <si>
+    <t>Same family compound</t>
+  </si>
+  <si>
+    <t>Virus isolation from acute-phase sera or pm liver fna samples; indirect IF on convalescent-phase sera</t>
+  </si>
+  <si>
+    <t>not direct contact</t>
+  </si>
+  <si>
+    <t>direct contact + nursing care</t>
+  </si>
+  <si>
+    <t>direct contact but NO nursing care</t>
+  </si>
+  <si>
+    <t>PMC2536234</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Henao-Restrepo</t>
+  </si>
+  <si>
+    <t>10.1016/ S0140-6736(16)32621-6</t>
+  </si>
+  <si>
+    <t>Basse-Guinée</t>
+  </si>
+  <si>
+    <t>Guinea</t>
+  </si>
+  <si>
+    <t>2015-2016</t>
+  </si>
+  <si>
+    <t>Zaire</t>
+  </si>
+  <si>
+    <t>Vaccine ring trial (delayed vaccination arm)</t>
+  </si>
+  <si>
+    <t>High-risk contacts were defined as being in close physical contact with the patient’s body or body fluids, linen, or clothes</t>
+  </si>
+  <si>
+    <t>high-risk</t>
+  </si>
+  <si>
+    <t>Laboratory-confirmed</t>
+  </si>
+  <si>
+    <t>10.1016/ S0140-6736(16)32621-7</t>
+  </si>
+  <si>
+    <t>As below - but not high risk...</t>
+  </si>
+  <si>
+    <t>non-high risk</t>
+  </si>
+  <si>
+    <t>10.1016/ S0140-6736(16)32621-8</t>
+  </si>
+  <si>
+    <t>Contacts were defined as individuals who lived in the same household, visited or were visited by the index case after the onset of symptoms, provided him or her with unprotected care, or prepared the body for the traditional funeral ceremony. </t>
+  </si>
+  <si>
+    <t>Jezek</t>
+  </si>
+  <si>
+    <t>10.1086/514293</t>
+  </si>
+  <si>
+    <t>Sud-Ubangi</t>
+  </si>
+  <si>
+    <t>DRC</t>
+  </si>
+  <si>
+    <t>1981-1983</t>
+  </si>
+  <si>
+    <t>Surveillance report</t>
+  </si>
+  <si>
+    <t>Provided care</t>
+  </si>
+  <si>
+    <t>IFA + clinical case definition</t>
+  </si>
+  <si>
+    <t>10.1086/514294</t>
+  </si>
+  <si>
+    <t>Did not provide care</t>
+  </si>
+  <si>
+    <t>10.1086/514295</t>
+  </si>
+  <si>
+    <t>A person who lived in the same house as the case patient or a non-household contact who had visited or cared for the case</t>
+  </si>
+  <si>
+    <t>Reichler</t>
+  </si>
+  <si>
+    <t>10.1093/infdis/jiy204</t>
+  </si>
+  <si>
+    <t>Freetown</t>
+  </si>
+  <si>
+    <t>Sierra Leone</t>
+  </si>
+  <si>
+    <t>2014-2015</t>
+  </si>
+  <si>
+    <t>Prospective</t>
+  </si>
+  <si>
+    <t>All household contacts</t>
+  </si>
+  <si>
+    <t>Defined household contacts as persons who spent at least 1 night sharing the same residential unit/indoor living space as the index case after their onset of symptoms. All index cases that died at home were removed for SDBs so there were no funeral/burial-related exposures.</t>
+  </si>
+  <si>
+    <t>Confirmed and probable secondary cases among contacts</t>
+  </si>
+  <si>
+    <t>10.1093/infdis/jiy205</t>
+  </si>
+  <si>
+    <t>Household contact who had direct physical contact with the index</t>
+  </si>
+  <si>
+    <t>10.1093/infdis/jiy206</t>
+  </si>
+  <si>
+    <t>Household contact with NO direct physical contact to index case</t>
+  </si>
+  <si>
+    <t>10.1093/infdis/jiy207</t>
+  </si>
+  <si>
+    <t>Household contact who provided nursing care (unprotected)</t>
+  </si>
+  <si>
+    <t>10.1093/infdis/jiy208</t>
+  </si>
+  <si>
+    <t>Household contact who provided nursing care with some protection</t>
+  </si>
+  <si>
+    <t>10.1093/infdis/jiy209</t>
+  </si>
+  <si>
+    <t>Household contact who did NOT provide nursing care</t>
+  </si>
+  <si>
+    <t>10.1093/infdis/jiy210</t>
+  </si>
+  <si>
+    <t>Household contact who had contact with index's body fluids </t>
+  </si>
+  <si>
+    <t>10.1093/infdis/jiy211</t>
+  </si>
+  <si>
+    <t>Household contact who did NOT have contact with body fluids</t>
+  </si>
+  <si>
+    <t>Francesconi</t>
+  </si>
+  <si>
+    <t>10.3201/eid0911.030339</t>
+  </si>
+  <si>
+    <t>Gulu District</t>
+  </si>
+  <si>
+    <t>Uganda</t>
+  </si>
+  <si>
+    <t>2000-2001</t>
+  </si>
+  <si>
+    <t>Sudan</t>
+  </si>
+  <si>
+    <t>Retrospective</t>
+  </si>
+  <si>
+    <t>A contact was defined as a person who had at least one of the following: 1) physical contact with case-patient (alive or dead), 2) slept in the same hut or house during the disease period, 3) contact with case-patient's body fluids during disease period, 4) contact with case-patient's linens or other possible fomites during disease or just after death.</t>
+  </si>
+  <si>
+    <t>10.3201/eid0911.030340</t>
+  </si>
+  <si>
+    <t>Contact as above + had direct physical contact</t>
+  </si>
+  <si>
+    <t>10.3201/eid0911.030341</t>
+  </si>
+  <si>
+    <t>Contact as above but did NOT have direct physical contact</t>
+  </si>
+  <si>
+    <t>10.3201/eid0911.030342</t>
+  </si>
+  <si>
+    <t>Contact as above + had contact with body fluids</t>
+  </si>
+  <si>
+    <t>10.3201/eid0911.030343</t>
+  </si>
+  <si>
+    <t>Contact as above but did NOT have contact with body fluids</t>
+  </si>
+  <si>
+    <t>10.3201/eid0911.030344</t>
+  </si>
+  <si>
+    <t>Contact as above + provided nursing care</t>
+  </si>
+  <si>
+    <t>10.3201/eid0911.030345</t>
+  </si>
+  <si>
+    <t>Contact as above but did NOT provide nursing care</t>
+  </si>
+  <si>
+    <t>Reaves</t>
+  </si>
+  <si>
+    <t>PMC5779472</t>
+  </si>
+  <si>
+    <t>Firestone District</t>
+  </si>
+  <si>
+    <t>Liberia</t>
+  </si>
+  <si>
+    <t>A contact was defined as a person with no symptoms who had physical contact with an Ebola patient or the body fluids of an Ebola patient within the past 21 days. Physical contact could be proven or highly suspected, such as having shared the same room or bed, cared for a patient, touched body fluids, or closely participated in a burial (e.g., physical contact with the corpse).</t>
+  </si>
+  <si>
+    <t>Not defined</t>
+  </si>
+  <si>
+    <t>PMC5779473</t>
+  </si>
+  <si>
+    <t>High-risk exposure identified as a percutaneous or mucous membrane exposure to, or direct skin contact with blood or body fluids of an Ebola patient or a corpse in Liberia without appropriate PPE</t>
+  </si>
+  <si>
+    <t>PMC5779474</t>
+  </si>
+  <si>
+    <t>Low-risk exposure defined as a household contact that did not involve providing care to an Ebola patient or having close contact with an Ebola patient in healthcare facilities or in the community that was not otherwise characterised as a high-risk exposure</t>
+  </si>
+  <si>
+    <t>low-risk</t>
+  </si>
+  <si>
+    <t>Dowell</t>
+  </si>
+  <si>
+    <t>disaggregated</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -177,8 +483,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -513,7 +821,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0DC51526-764C-BF40-8961-705EA21594C9}">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="14.6640625" bestFit="1" customWidth="1"/>
@@ -525,61 +833,1659 @@
     <col min="15" max="15" width="13.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1983</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="2">
+        <v>1979</v>
+      </c>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J2" s="2">
+        <v>9</v>
+      </c>
+      <c r="K2" s="2">
+        <v>1</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M2" s="2">
+        <v>27</v>
+      </c>
+      <c r="N2" s="2">
+        <v>86</v>
+      </c>
+      <c r="O2" s="2">
+        <v>132</v>
+      </c>
+      <c r="P2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1983</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1979</v>
+      </c>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J3" s="2">
+        <v>9</v>
+      </c>
+      <c r="K3" s="2">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M3" s="2">
+        <v>0</v>
+      </c>
+      <c r="N3" s="2">
+        <v>44</v>
+      </c>
+      <c r="O3" s="2">
+        <v>132</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1983</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="2">
+        <v>1979</v>
+      </c>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="J4" s="2">
+        <v>9</v>
+      </c>
+      <c r="K4" s="2">
+        <v>1</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M4" s="2">
+        <v>24</v>
+      </c>
+      <c r="N4" s="2">
+        <v>60</v>
+      </c>
+      <c r="O4" s="2">
+        <v>132</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1983</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="2">
+        <v>1979</v>
+      </c>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="J5" s="2">
+        <v>9</v>
+      </c>
+      <c r="K5" s="2">
+        <v>1</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M5" s="2">
+        <v>3</v>
+      </c>
+      <c r="N5" s="2">
+        <v>26</v>
+      </c>
+      <c r="O5" s="2">
+        <v>132</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q5" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1983</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="2">
+        <v>1979</v>
+      </c>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="J6" s="2">
+        <v>9</v>
+      </c>
+      <c r="K6" s="2">
+        <v>1</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M6" s="2">
+        <v>29</v>
+      </c>
+      <c r="N6" s="2">
+        <v>132</v>
+      </c>
+      <c r="O6" s="2">
+        <v>132</v>
+      </c>
+      <c r="P6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="Q6" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="2">
+        <v>2017</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="K7" s="2">
+        <v>2</v>
+      </c>
+      <c r="L7" s="2">
+        <v>9</v>
+      </c>
+      <c r="M7" s="2">
+        <v>6</v>
+      </c>
+      <c r="N7" s="2">
+        <v>231</v>
+      </c>
+      <c r="O7" s="2">
+        <v>412</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B8" s="2">
+        <v>2017</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="K8" s="2">
+        <v>2</v>
+      </c>
+      <c r="L8" s="2">
+        <v>9</v>
+      </c>
+      <c r="M8" s="2">
+        <v>7</v>
+      </c>
+      <c r="N8" s="2">
+        <v>181</v>
+      </c>
+      <c r="O8" s="2">
+        <v>412</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q8" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="2">
+        <v>2017</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="J9" s="2">
+        <v>9</v>
+      </c>
+      <c r="K9" s="2">
+        <v>2</v>
+      </c>
+      <c r="L9" s="2">
+        <v>9</v>
+      </c>
+      <c r="M9" s="2">
+        <v>13</v>
+      </c>
+      <c r="N9" s="2">
+        <v>412</v>
+      </c>
+      <c r="O9" s="2">
+        <v>412</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="Q9" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B10" s="2">
+        <v>1999</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="J10" s="2">
+        <v>9</v>
+      </c>
+      <c r="K10" s="2">
+        <v>2</v>
+      </c>
+      <c r="L10" s="2">
+        <v>9</v>
+      </c>
+      <c r="M10" s="2">
+        <v>9</v>
+      </c>
+      <c r="N10" s="2">
+        <v>51</v>
+      </c>
+      <c r="O10" s="2">
+        <v>188</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="2">
+        <v>1999</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="J11" s="2">
+        <v>9</v>
+      </c>
+      <c r="K11" s="2">
+        <v>2</v>
+      </c>
+      <c r="L11" s="2">
+        <v>9</v>
+      </c>
+      <c r="M11" s="2">
+        <v>19</v>
+      </c>
+      <c r="N11" s="2">
+        <v>137</v>
+      </c>
+      <c r="O11" s="2">
+        <v>188</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="2">
+        <v>1999</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="J12" s="2">
+        <v>9</v>
+      </c>
+      <c r="K12" s="2">
+        <v>2</v>
+      </c>
+      <c r="L12" s="2">
+        <v>9</v>
+      </c>
+      <c r="M12" s="2">
+        <v>28</v>
+      </c>
+      <c r="N12" s="2">
+        <v>188</v>
+      </c>
+      <c r="O12" s="2">
+        <v>188</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B13" s="2">
+        <v>2018</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="J13" s="2">
+        <v>9</v>
+      </c>
+      <c r="K13" s="2">
+        <v>1</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M13" s="2">
+        <v>83</v>
+      </c>
+      <c r="N13" s="2">
+        <v>838</v>
+      </c>
+      <c r="O13" s="2">
+        <v>838</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>9</v>
+      </c>
+      <c r="R13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" s="2">
+        <v>2018</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="J14" s="2">
+        <v>9</v>
+      </c>
+      <c r="K14" s="2">
+        <v>1</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M14" s="2">
+        <v>50</v>
+      </c>
+      <c r="N14" s="2">
+        <v>289</v>
+      </c>
+      <c r="O14" s="2">
+        <v>838</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>9</v>
+      </c>
+      <c r="R14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B15" s="2">
+        <v>2018</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="J15" s="2">
+        <v>9</v>
+      </c>
+      <c r="K15" s="2">
+        <v>1</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M15" s="2">
+        <v>33</v>
+      </c>
+      <c r="N15" s="2">
+        <v>548</v>
+      </c>
+      <c r="O15" s="2">
+        <v>838</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>9</v>
+      </c>
+      <c r="R15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A16" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B16" s="2">
+        <v>2018</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="J16" s="2">
+        <v>9</v>
+      </c>
+      <c r="K16" s="2">
+        <v>1</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M16" s="2">
+        <v>32</v>
+      </c>
+      <c r="N16" s="2">
+        <v>134</v>
+      </c>
+      <c r="O16" s="2">
+        <v>838</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>9</v>
+      </c>
+      <c r="R16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A17" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B17" s="2">
+        <v>2018</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="J17" s="2">
+        <v>9</v>
+      </c>
+      <c r="K17" s="2">
+        <v>1</v>
+      </c>
+      <c r="L17" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M17" s="2">
+        <v>5</v>
+      </c>
+      <c r="N17" s="2">
+        <v>22</v>
+      </c>
+      <c r="O17" s="2">
+        <v>838</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>9</v>
+      </c>
+      <c r="R17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A18" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B18" s="2">
+        <v>2018</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="J18" s="2">
+        <v>9</v>
+      </c>
+      <c r="K18" s="2">
+        <v>1</v>
+      </c>
+      <c r="L18" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M18" s="2">
+        <v>46</v>
+      </c>
+      <c r="N18" s="2">
+        <v>682</v>
+      </c>
+      <c r="O18" s="2">
+        <v>838</v>
+      </c>
+      <c r="P18" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q18" s="2">
+        <v>9</v>
+      </c>
+      <c r="R18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A19" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B19" s="2">
+        <v>2018</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="J19" s="2">
+        <v>9</v>
+      </c>
+      <c r="K19" s="2">
+        <v>1</v>
+      </c>
+      <c r="L19" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M19" s="2">
+        <v>24</v>
+      </c>
+      <c r="N19" s="2">
+        <v>112</v>
+      </c>
+      <c r="O19" s="2">
+        <v>838</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>9</v>
+      </c>
+      <c r="R19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A20" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" s="2">
+        <v>2018</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="J20" s="2">
+        <v>9</v>
+      </c>
+      <c r="K20" s="2">
+        <v>1</v>
+      </c>
+      <c r="L20" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="M20" s="2">
+        <v>56</v>
+      </c>
+      <c r="N20" s="2">
+        <v>718</v>
+      </c>
+      <c r="O20" s="2">
+        <v>838</v>
+      </c>
+      <c r="P20" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q20" s="2">
+        <v>9</v>
+      </c>
+      <c r="R20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A21" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B21" s="2">
+        <v>2003</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="J21" s="2">
+        <v>9</v>
+      </c>
+      <c r="K21" s="2">
+        <v>2</v>
+      </c>
+      <c r="L21" s="2">
+        <v>9</v>
+      </c>
+      <c r="M21" s="2">
+        <v>24</v>
+      </c>
+      <c r="N21" s="2">
+        <v>89</v>
+      </c>
+      <c r="O21" s="2">
+        <v>89</v>
+      </c>
+      <c r="P21" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q21" s="2">
+        <v>9</v>
+      </c>
+      <c r="R21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A22" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B22" s="2">
+        <v>2003</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J22" s="2">
+        <v>9</v>
+      </c>
+      <c r="K22" s="2">
+        <v>2</v>
+      </c>
+      <c r="L22" s="2">
+        <v>9</v>
+      </c>
+      <c r="M22" s="2">
+        <v>19</v>
+      </c>
+      <c r="N22" s="2">
+        <v>70</v>
+      </c>
+      <c r="O22" s="2">
+        <v>89</v>
+      </c>
+      <c r="P22" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>9</v>
+      </c>
+      <c r="R22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B23" s="2">
+        <v>2003</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="J23" s="2">
+        <v>9</v>
+      </c>
+      <c r="K23" s="2">
+        <v>2</v>
+      </c>
+      <c r="L23" s="2">
+        <v>9</v>
+      </c>
+      <c r="M23" s="2">
+        <v>1</v>
+      </c>
+      <c r="N23" s="2">
+        <v>13</v>
+      </c>
+      <c r="O23" s="2">
+        <v>89</v>
+      </c>
+      <c r="P23" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q23" s="2">
+        <v>9</v>
+      </c>
+      <c r="R23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A24" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B24" s="2">
+        <v>2003</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="J24" s="2">
+        <v>9</v>
+      </c>
+      <c r="K24" s="2">
+        <v>2</v>
+      </c>
+      <c r="L24" s="2">
+        <v>9</v>
+      </c>
+      <c r="M24" s="2">
+        <v>15</v>
+      </c>
+      <c r="N24" s="2">
+        <v>30</v>
+      </c>
+      <c r="O24" s="2">
+        <v>89</v>
+      </c>
+      <c r="P24" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>9</v>
+      </c>
+      <c r="R24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A25" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B25" s="2">
+        <v>2003</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="J25" s="2">
+        <v>9</v>
+      </c>
+      <c r="K25" s="2">
+        <v>2</v>
+      </c>
+      <c r="L25" s="2">
+        <v>9</v>
+      </c>
+      <c r="M25" s="2">
+        <v>5</v>
+      </c>
+      <c r="N25" s="2">
+        <v>53</v>
+      </c>
+      <c r="O25" s="2">
+        <v>89</v>
+      </c>
+      <c r="P25" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q25" s="2">
+        <v>9</v>
+      </c>
+      <c r="R25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A26" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B26" s="2">
+        <v>2003</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="J26" s="2">
+        <v>9</v>
+      </c>
+      <c r="K26" s="2">
+        <v>2</v>
+      </c>
+      <c r="L26" s="2">
+        <v>9</v>
+      </c>
+      <c r="M26" s="2">
+        <v>2</v>
+      </c>
+      <c r="N26" s="2">
+        <v>40</v>
+      </c>
+      <c r="O26" s="2">
+        <v>89</v>
+      </c>
+      <c r="P26" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q26" s="2">
+        <v>9</v>
+      </c>
+      <c r="R26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A27" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B27" s="2">
+        <v>2003</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="J27" s="2">
+        <v>9</v>
+      </c>
+      <c r="K27" s="2">
+        <v>2</v>
+      </c>
+      <c r="L27" s="2">
+        <v>9</v>
+      </c>
+      <c r="M27" s="2">
+        <v>18</v>
+      </c>
+      <c r="N27" s="2">
+        <v>43</v>
+      </c>
+      <c r="O27" s="2">
+        <v>89</v>
+      </c>
+      <c r="P27" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="Q27" s="2">
+        <v>9</v>
+      </c>
+      <c r="R27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A28" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B28" s="2">
+        <v>2014</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F28" s="2">
+        <v>2014</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="J28" s="2">
+        <v>9</v>
+      </c>
+      <c r="K28" s="2">
+        <v>2</v>
+      </c>
+      <c r="L28" s="2">
+        <v>9</v>
+      </c>
+      <c r="M28" s="2">
         <v>21</v>
       </c>
-      <c r="I1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" t="s">
-        <v>11</v>
-      </c>
-      <c r="L1" t="s">
-        <v>12</v>
-      </c>
-      <c r="M1" t="s">
-        <v>9</v>
-      </c>
-      <c r="N1" t="s">
-        <v>10</v>
-      </c>
-      <c r="O1" t="s">
-        <v>13</v>
-      </c>
+      <c r="N28" s="2">
+        <v>233</v>
+      </c>
+      <c r="O28" s="2">
+        <v>233</v>
+      </c>
+      <c r="P28" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A29" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B29" s="2">
+        <v>2014</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F29" s="2">
+        <v>2014</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="K29" s="2">
+        <v>2</v>
+      </c>
+      <c r="L29" s="2">
+        <v>9</v>
+      </c>
+      <c r="M29" s="2">
+        <v>21</v>
+      </c>
+      <c r="N29" s="2">
+        <v>74</v>
+      </c>
+      <c r="O29" s="2">
+        <v>233</v>
+      </c>
+      <c r="P29" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q29" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A30" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B30" s="2">
+        <v>2014</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="F30" s="2">
+        <v>2014</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="K30" s="2">
+        <v>2</v>
+      </c>
+      <c r="L30" s="2">
+        <v>9</v>
+      </c>
+      <c r="M30" s="2">
+        <v>0</v>
+      </c>
+      <c r="N30" s="2">
+        <v>159</v>
+      </c>
+      <c r="O30" s="2">
+        <v>233</v>
+      </c>
+      <c r="P30" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q30" s="2">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A31" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B31" s="2">
+        <v>1999</v>
+      </c>
+      <c r="C31" s="2"/>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2"/>
+      <c r="J31" s="2"/>
+      <c r="K31" s="2"/>
+      <c r="L31" s="2"/>
+      <c r="M31" s="2"/>
+      <c r="N31" s="2"/>
+      <c r="O31" s="2"/>
+      <c r="P31" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D66B454-BB03-3B4F-ACCC-AB275053BB74}">
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="18.1640625" bestFit="1" customWidth="1"/>
@@ -623,7 +2529,7 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -631,7 +2537,7 @@
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>20</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
@@ -639,7 +2545,7 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -647,15 +2553,15 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
@@ -663,7 +2569,7 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
@@ -671,7 +2577,7 @@
         <v>8</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
@@ -679,7 +2585,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -687,7 +2593,7 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
@@ -695,7 +2601,7 @@
         <v>9</v>
       </c>
       <c r="B14" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
@@ -703,23 +2609,31 @@
         <v>10</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>13</v>
       </c>
-      <c r="B17" t="s">
-        <v>33</v>
+      <c r="B18" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>